<commit_message>
City index 26-03 11/11 final
</commit_message>
<xml_diff>
--- a/data_indexpoints_tidy/tallmateriale_19954.xlsx
+++ b/data_indexpoints_tidy/tallmateriale_19954.xlsx
@@ -1372,6 +1372,9 @@
       <c r="F3">
         <v>3.17</v>
       </c>
+      <c r="G3">
+        <v>5.49</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1445,6 +1448,9 @@
       <c r="F5">
         <v>4.24</v>
       </c>
+      <c r="G5">
+        <v>4.55</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1527,6 +1533,9 @@
       <c r="F7">
         <v>3.03</v>
       </c>
+      <c r="G7">
+        <v>3.43</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1597,6 +1606,9 @@
       <c r="F9">
         <v>-1.02</v>
       </c>
+      <c r="G9">
+        <v>2.76</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1679,6 +1691,9 @@
       <c r="F11">
         <v>-0.74</v>
       </c>
+      <c r="G11">
+        <v>0.6899999999999999</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1761,6 +1776,9 @@
       <c r="F13">
         <v>3.01</v>
       </c>
+      <c r="G13">
+        <v>5.49</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1843,6 +1861,9 @@
       <c r="F15">
         <v>5.2</v>
       </c>
+      <c r="G15">
+        <v>4.81</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1925,6 +1946,9 @@
       <c r="F17">
         <v>6.69</v>
       </c>
+      <c r="G17">
+        <v>7.73</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2007,6 +2031,9 @@
       <c r="F19">
         <v>6.06</v>
       </c>
+      <c r="G19">
+        <v>7.53</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2152,6 +2179,9 @@
       </c>
       <c r="F23">
         <v>-2.46</v>
+      </c>
+      <c r="G23">
+        <v>-2.44</v>
       </c>
     </row>
   </sheetData>
@@ -2298,19 +2328,19 @@
         <v>2026</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="E3">
-        <v>1.0265</v>
+        <v>1.032</v>
       </c>
       <c r="F3">
         <v>10</v>
       </c>
       <c r="G3">
-        <v>0.9689646843432461</v>
+        <v>0.9878107732945247</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -2329,19 +2359,19 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>feb</t>
+          <t>mar</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>jan-feb</t>
+          <t>jan-mar</t>
         </is>
       </c>
       <c r="M3">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="N3">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
     </row>
   </sheetData>
@@ -2434,19 +2464,19 @@
         <v>2025</v>
       </c>
       <c r="C2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D2">
-        <v>3.3</v>
+        <v>4.3</v>
       </c>
       <c r="E2">
-        <v>1.0331</v>
+        <v>1.0435</v>
       </c>
       <c r="F2">
         <v>11</v>
       </c>
       <c r="G2">
-        <v>0.8430676316018484</v>
+        <v>0.8465321606646595</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -2465,19 +2495,19 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>feb</t>
+          <t>mar</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>jan-feb</t>
+          <t>jan-mar</t>
         </is>
       </c>
       <c r="M2">
-        <v>1.6</v>
+        <v>2.6</v>
       </c>
       <c r="N2">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -2488,19 +2518,19 @@
         <v>2026</v>
       </c>
       <c r="C3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
       <c r="E3">
-        <v>1.0265</v>
+        <v>1.032</v>
       </c>
       <c r="F3">
         <v>10</v>
       </c>
       <c r="G3">
-        <v>0.9689646843432461</v>
+        <v>0.9878107732945247</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -2519,19 +2549,19 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>feb</t>
+          <t>mar</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>jan-feb</t>
+          <t>jan-mar</t>
         </is>
       </c>
       <c r="M3">
-        <v>0.7</v>
+        <v>1.3</v>
       </c>
       <c r="N3">
-        <v>4.5</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="4">
@@ -2542,19 +2572,19 @@
         <v>2026</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>7.7</v>
       </c>
       <c r="E4">
-        <v>1.06047715</v>
+        <v>1.076892</v>
       </c>
       <c r="F4">
         <v>11</v>
       </c>
       <c r="G4">
-        <v>1.323281997721419</v>
+        <v>1.351218869843741</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -2573,19 +2603,19 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>feb</t>
+          <t>mar</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>jan-feb</t>
+          <t>jan-mar</t>
         </is>
       </c>
       <c r="M4">
-        <v>3.4</v>
+        <v>5.1</v>
       </c>
       <c r="N4">
-        <v>8.6</v>
+        <v>10.3</v>
       </c>
     </row>
   </sheetData>
@@ -2595,7 +2625,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="10" max="10" width="20.7109375" style="2" customWidth="1"/>
@@ -2803,6 +2833,51 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5">
+        <v>1.042643039966005</v>
+      </c>
+      <c r="B5">
+        <v>4.264303996600494</v>
+      </c>
+      <c r="C5">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>6.961550277176276</v>
+      </c>
+      <c r="E5">
+        <v>3.453201038408007</v>
+      </c>
+      <c r="F5">
+        <v>1.308786723552142</v>
+      </c>
+      <c r="G5">
+        <v>1.2</v>
+      </c>
+      <c r="H5">
+        <v>7.4</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2024 - (apr 2025 - mar 2026)</t>
+        </is>
+      </c>
+      <c r="J5" s="2">
+        <v>46082</v>
+      </c>
+      <c r="K5">
+        <v>3</v>
+      </c>
+      <c r="L5">
+        <v>2026</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>12_months</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
City index 26-7 11/11.
</commit_message>
<xml_diff>
--- a/data_indexpoints_tidy/tallmateriale_19954.xlsx
+++ b/data_indexpoints_tidy/tallmateriale_19954.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Programmering\R\byindeks\data_indexpoints_tidy\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E906A89-1A5D-4D04-9003-A68C40C9CE26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="20985" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="punkt_adt" sheetId="1" r:id="rId1"/>
@@ -19,12 +13,12 @@
     <sheet name="byindeks_hittil" sheetId="4" r:id="rId4"/>
     <sheet name="by_glid_indeks" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="112">
   <si>
     <t>trp_id</t>
   </si>
@@ -254,64 +248,76 @@
     <t>des</t>
   </si>
   <si>
+    <t>area_name</t>
+  </si>
+  <si>
     <t>year_base</t>
   </si>
   <si>
+    <t>year_from_to</t>
+  </si>
+  <si>
     <t>month</t>
   </si>
   <si>
+    <t>month_name_short</t>
+  </si>
+  <si>
+    <t>period</t>
+  </si>
+  <si>
+    <t>index_type</t>
+  </si>
+  <si>
+    <t>n_trp</t>
+  </si>
+  <si>
+    <t>index_i</t>
+  </si>
+  <si>
     <t>index_p</t>
   </si>
   <si>
-    <t>index_i</t>
-  </si>
-  <si>
-    <t>n_trp</t>
-  </si>
-  <si>
     <t>standard_error</t>
   </si>
   <si>
-    <t>index_type</t>
-  </si>
-  <si>
-    <t>year_from_to</t>
-  </si>
-  <si>
-    <t>area_name</t>
-  </si>
-  <si>
-    <t>month_name_short</t>
-  </si>
-  <si>
-    <t>period</t>
-  </si>
-  <si>
     <t>ci_lower</t>
   </si>
   <si>
     <t>ci_upper</t>
   </si>
   <si>
+    <t>2024-2025</t>
+  </si>
+  <si>
+    <t>jan-des</t>
+  </si>
+  <si>
     <t>direct</t>
   </si>
   <si>
-    <t>2024-2025</t>
-  </si>
-  <si>
-    <t>jan-des</t>
-  </si>
-  <si>
     <t>2025-2026</t>
   </si>
   <si>
-    <t>jan-apr</t>
+    <t>jan-jul</t>
+  </si>
+  <si>
+    <t>2024-2026</t>
   </si>
   <si>
     <t>chained</t>
   </si>
   <si>
-    <t>2024-2026</t>
+    <t>month_n</t>
+  </si>
+  <si>
+    <t>month_object</t>
+  </si>
+  <si>
+    <t>window</t>
+  </si>
+  <si>
+    <t>index_period</t>
   </si>
   <si>
     <t>n_eff</t>
@@ -323,24 +329,12 @@
     <t>standard_error_p</t>
   </si>
   <si>
-    <t>index_period</t>
-  </si>
-  <si>
-    <t>month_object</t>
-  </si>
-  <si>
-    <t>month_n</t>
-  </si>
-  <si>
-    <t>window</t>
+    <t>12_months</t>
   </si>
   <si>
     <t>2024 - (jan 2025 - des 2025)</t>
   </si>
   <si>
-    <t>12_months</t>
-  </si>
-  <si>
     <t>2024 - (feb 2025 - jan 2026)</t>
   </si>
   <si>
@@ -351,16 +345,25 @@
   </si>
   <si>
     <t>2024 - (mai 2025 - apr 2026)</t>
+  </si>
+  <si>
+    <t>2024 - (jun 2025 - mai 2026)</t>
+  </si>
+  <si>
+    <t>2024 - (jul 2025 - jun 2026)</t>
+  </si>
+  <si>
+    <t>2024 - (aug 2025 - jul 2026)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -409,21 +412,13 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -461,7 +456,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -495,7 +490,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -530,10 +524,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -706,11 +699,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P12"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -760,7 +753,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -777,10 +770,10 @@
         <v>20</v>
       </c>
       <c r="F2">
-        <v>67.288186999999994</v>
+        <v>67.28818699999999</v>
       </c>
       <c r="G2">
-        <v>14.420325999999999</v>
+        <v>14.420326</v>
       </c>
       <c r="H2" t="s">
         <v>21</v>
@@ -807,7 +800,7 @@
         <v>450</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -824,7 +817,7 @@
         <v>20</v>
       </c>
       <c r="F3">
-        <v>67.281290999999996</v>
+        <v>67.281291</v>
       </c>
       <c r="G3">
         <v>14.46311</v>
@@ -842,10 +835,10 @@
         <v>5860</v>
       </c>
       <c r="M3">
-        <v>6630</v>
+        <v>8010</v>
       </c>
       <c r="N3">
-        <v>670</v>
+        <v>820</v>
       </c>
       <c r="O3">
         <v>8230</v>
@@ -854,7 +847,7 @@
         <v>830</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -871,10 +864,10 @@
         <v>20</v>
       </c>
       <c r="F4">
-        <v>67.281497000000002</v>
+        <v>67.281497</v>
       </c>
       <c r="G4">
-        <v>14.463013999999999</v>
+        <v>14.463014</v>
       </c>
       <c r="H4" t="s">
         <v>30</v>
@@ -889,10 +882,10 @@
         <v>5950</v>
       </c>
       <c r="M4">
-        <v>6670</v>
+        <v>8060</v>
       </c>
       <c r="N4">
-        <v>620</v>
+        <v>750</v>
       </c>
       <c r="O4">
         <v>8220</v>
@@ -901,7 +894,7 @@
         <v>850</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>31</v>
       </c>
@@ -918,10 +911,10 @@
         <v>20</v>
       </c>
       <c r="F5">
-        <v>67.278277000000003</v>
+        <v>67.278277</v>
       </c>
       <c r="G5">
-        <v>14.516923999999999</v>
+        <v>14.516924</v>
       </c>
       <c r="H5" t="s">
         <v>34</v>
@@ -948,7 +941,7 @@
         <v>2060</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -995,7 +988,7 @@
         <v>2020</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>39</v>
       </c>
@@ -1012,7 +1005,7 @@
         <v>20</v>
       </c>
       <c r="F7">
-        <v>67.283801999999994</v>
+        <v>67.28380199999999</v>
       </c>
       <c r="G7">
         <v>14.558532</v>
@@ -1042,7 +1035,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>43</v>
       </c>
@@ -1059,7 +1052,7 @@
         <v>20</v>
       </c>
       <c r="F8">
-        <v>67.273696999999999</v>
+        <v>67.273697</v>
       </c>
       <c r="G8">
         <v>14.37946</v>
@@ -1089,7 +1082,7 @@
         <v>1300</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16">
       <c r="A9" t="s">
         <v>47</v>
       </c>
@@ -1106,7 +1099,7 @@
         <v>20</v>
       </c>
       <c r="F9">
-        <v>67.274722999999994</v>
+        <v>67.27472299999999</v>
       </c>
       <c r="G9">
         <v>14.397437</v>
@@ -1136,7 +1129,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -1153,10 +1146,10 @@
         <v>20</v>
       </c>
       <c r="F10">
-        <v>67.277069999999995</v>
+        <v>67.27706999999999</v>
       </c>
       <c r="G10">
-        <v>14.429798999999999</v>
+        <v>14.429799</v>
       </c>
       <c r="H10" t="s">
         <v>54</v>
@@ -1183,7 +1176,7 @@
         <v>1560</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
         <v>55</v>
       </c>
@@ -1200,10 +1193,10 @@
         <v>20</v>
       </c>
       <c r="F11">
-        <v>67.286271999999997</v>
+        <v>67.286272</v>
       </c>
       <c r="G11">
-        <v>14.397085000000001</v>
+        <v>14.397085</v>
       </c>
       <c r="H11" t="s">
         <v>58</v>
@@ -1230,7 +1223,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16">
       <c r="A12" t="s">
         <v>59</v>
       </c>
@@ -1247,7 +1240,7 @@
         <v>20</v>
       </c>
       <c r="F12">
-        <v>67.282331999999997</v>
+        <v>67.282332</v>
       </c>
       <c r="G12">
         <v>14.417163</v>
@@ -1283,11 +1276,11 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:P23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1337,7 +1330,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>22</v>
       </c>
@@ -1351,7 +1344,7 @@
         <v>2025</v>
       </c>
       <c r="E2">
-        <v>2.4500000000000002</v>
+        <v>2.45</v>
       </c>
       <c r="F2">
         <v>4.03</v>
@@ -1360,7 +1353,7 @@
         <v>6.53</v>
       </c>
       <c r="H2">
-        <v>-8.4499999999999993</v>
+        <v>-8.449999999999999</v>
       </c>
       <c r="I2">
         <v>1.25</v>
@@ -1378,7 +1371,7 @@
         <v>6.12</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>22</v>
       </c>
@@ -1403,8 +1396,17 @@
       <c r="H3">
         <v>6.73</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I3">
+        <v>-0.1</v>
+      </c>
+      <c r="J3">
+        <v>1.01</v>
+      </c>
+      <c r="K3">
+        <v>-2.26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -1445,7 +1447,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1470,8 +1472,17 @@
       <c r="H5">
         <v>7.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I5">
+        <v>0.36</v>
+      </c>
+      <c r="J5">
+        <v>1.17</v>
+      </c>
+      <c r="K5">
+        <v>-2.17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
         <v>31</v>
       </c>
@@ -1509,7 +1520,7 @@
         <v>2.37</v>
       </c>
       <c r="M6">
-        <v>2.4900000000000002</v>
+        <v>2.49</v>
       </c>
       <c r="N6">
         <v>2.99</v>
@@ -1518,10 +1529,10 @@
         <v>1.27</v>
       </c>
       <c r="P6">
-        <v>5.0199999999999996</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+        <v>5.02</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -1546,8 +1557,17 @@
       <c r="H7">
         <v>7.23</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I7">
+        <v>-0.43</v>
+      </c>
+      <c r="J7">
+        <v>1.8</v>
+      </c>
+      <c r="K7">
+        <v>-3.28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -1567,7 +1587,7 @@
         <v>9.57</v>
       </c>
       <c r="K8">
-        <v>19.010000000000002</v>
+        <v>19.01</v>
       </c>
       <c r="L8">
         <v>13.18</v>
@@ -1585,7 +1605,7 @@
         <v>11.85</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -1610,8 +1630,17 @@
       <c r="H9">
         <v>7.92</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I9">
+        <v>-7.07</v>
+      </c>
+      <c r="J9">
+        <v>-4.45</v>
+      </c>
+      <c r="K9">
+        <v>-12.55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1661,7 +1690,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -1675,19 +1704,28 @@
         <v>2026</v>
       </c>
       <c r="E11">
-        <v>-1.1200000000000001</v>
+        <v>-1.12</v>
       </c>
       <c r="F11">
         <v>-0.74</v>
       </c>
       <c r="G11">
-        <v>0.69</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="H11">
         <v>5.71</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I11">
+        <v>-0.79</v>
+      </c>
+      <c r="J11">
+        <v>3.08</v>
+      </c>
+      <c r="K11">
+        <v>-5.95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -1722,7 +1760,7 @@
         <v>4.91</v>
       </c>
       <c r="L12">
-        <v>4.8099999999999996</v>
+        <v>4.81</v>
       </c>
       <c r="M12">
         <v>4.41</v>
@@ -1737,7 +1775,7 @@
         <v>7.11</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -1751,7 +1789,7 @@
         <v>2026</v>
       </c>
       <c r="E13">
-        <v>4.6100000000000003</v>
+        <v>4.61</v>
       </c>
       <c r="F13">
         <v>3.01</v>
@@ -1762,8 +1800,17 @@
       <c r="H13">
         <v>6.72</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I13">
+        <v>-1.12</v>
+      </c>
+      <c r="J13">
+        <v>1.21</v>
+      </c>
+      <c r="K13">
+        <v>-5.39</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
       <c r="A14" t="s">
         <v>43</v>
       </c>
@@ -1795,10 +1842,10 @@
         <v>0.92</v>
       </c>
       <c r="K14">
-        <v>-2.5299999999999998</v>
+        <v>-2.53</v>
       </c>
       <c r="L14">
-        <v>-0.14000000000000001</v>
+        <v>-0.14</v>
       </c>
       <c r="M14">
         <v>-1.51</v>
@@ -1813,7 +1860,7 @@
         <v>-1.05</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:16">
       <c r="A15" t="s">
         <v>43</v>
       </c>
@@ -1827,19 +1874,28 @@
         <v>2026</v>
       </c>
       <c r="E15">
-        <v>0.57999999999999996</v>
+        <v>0.58</v>
       </c>
       <c r="F15">
         <v>5.2</v>
       </c>
       <c r="G15">
-        <v>4.8099999999999996</v>
+        <v>4.81</v>
       </c>
       <c r="H15">
         <v>6.67</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I15">
+        <v>4.53</v>
+      </c>
+      <c r="J15">
+        <v>9.640000000000001</v>
+      </c>
+      <c r="K15">
+        <v>9.75</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
       <c r="A16" t="s">
         <v>47</v>
       </c>
@@ -1865,7 +1921,7 @@
         <v>-3.34</v>
       </c>
       <c r="I16">
-        <v>8.2100000000000009</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="J16">
         <v>9.66</v>
@@ -1874,10 +1930,10 @@
         <v>7.36</v>
       </c>
       <c r="L16">
-        <v>8.86</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="M16">
-        <v>9.3699999999999992</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="N16">
         <v>5.29</v>
@@ -1889,7 +1945,7 @@
         <v>11.11</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:16">
       <c r="A17" t="s">
         <v>47</v>
       </c>
@@ -1914,8 +1970,17 @@
       <c r="H17">
         <v>7.24</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I17">
+        <v>2.07</v>
+      </c>
+      <c r="J17">
+        <v>6.02</v>
+      </c>
+      <c r="K17">
+        <v>2.77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -1947,10 +2012,10 @@
         <v>9.66</v>
       </c>
       <c r="K18">
-        <v>8.89</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="L18">
-        <v>8.6999999999999993</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="M18">
         <v>9.42</v>
@@ -1962,10 +2027,10 @@
         <v>5.42</v>
       </c>
       <c r="P18">
-        <v>9.9600000000000009</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+        <v>9.960000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16">
       <c r="A19" t="s">
         <v>51</v>
       </c>
@@ -1990,8 +2055,17 @@
       <c r="H19">
         <v>8.08</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>2.96</v>
+      </c>
+      <c r="K19">
+        <v>-7.43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -2008,13 +2082,13 @@
         <v>3.03</v>
       </c>
       <c r="F20">
-        <v>2.2200000000000002</v>
+        <v>2.22</v>
       </c>
       <c r="G20">
         <v>1.33</v>
       </c>
       <c r="H20">
-        <v>-18.149999999999999</v>
+        <v>-18.15</v>
       </c>
       <c r="I20">
         <v>-4.82</v>
@@ -2029,7 +2103,7 @@
         <v>-24.47</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:16">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -2043,7 +2117,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:16">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -2075,25 +2149,25 @@
         <v>-1.03</v>
       </c>
       <c r="K22">
-        <v>-2.4300000000000002</v>
+        <v>-2.43</v>
       </c>
       <c r="L22">
         <v>-2.09</v>
       </c>
       <c r="M22">
-        <v>1.1599999999999999</v>
+        <v>1.16</v>
       </c>
       <c r="N22">
         <v>3.56</v>
       </c>
       <c r="O22">
-        <v>-4.2300000000000004</v>
+        <v>-4.23</v>
       </c>
       <c r="P22">
         <v>-3.97</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:16">
       <c r="A23" t="s">
         <v>59</v>
       </c>
@@ -2116,7 +2190,16 @@
         <v>-2.44</v>
       </c>
       <c r="H23">
-        <v>2.4900000000000002</v>
+        <v>2.49</v>
+      </c>
+      <c r="I23">
+        <v>-4.98</v>
+      </c>
+      <c r="J23">
+        <v>-0.39</v>
+      </c>
+      <c r="K23">
+        <v>-4.08</v>
       </c>
     </row>
   </sheetData>
@@ -2125,19 +2208,19 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>78</v>
@@ -2173,92 +2256,92 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
         <v>2024</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>2025</v>
       </c>
-      <c r="C2">
+      <c r="D2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E2">
         <v>12</v>
       </c>
-      <c r="D2">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="E2">
+      <c r="F2" t="s">
+        <v>75</v>
+      </c>
+      <c r="G2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I2">
+        <v>11</v>
+      </c>
+      <c r="J2">
         <v>1.0224</v>
       </c>
-      <c r="F2">
-        <v>11</v>
-      </c>
-      <c r="G2">
-        <v>1.5998620850388581</v>
-      </c>
-      <c r="H2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J2" t="s">
-        <v>20</v>
-      </c>
-      <c r="K2" t="s">
-        <v>75</v>
-      </c>
-      <c r="L2" t="s">
-        <v>91</v>
+      <c r="K2">
+        <v>2.24</v>
+      </c>
+      <c r="L2">
+        <v>1.599862085038858</v>
       </c>
       <c r="M2">
         <v>-0.9</v>
       </c>
       <c r="N2">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3">
+        <v>5.38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3">
         <v>2025</v>
       </c>
-      <c r="B3">
+      <c r="C3">
         <v>2026</v>
       </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>4.0999999999999996</v>
+      <c r="D3" t="s">
+        <v>92</v>
       </c>
       <c r="E3">
-        <v>1.0407999999999999</v>
-      </c>
-      <c r="F3">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" t="s">
+        <v>93</v>
+      </c>
+      <c r="H3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3">
         <v>10</v>
       </c>
-      <c r="G3">
-        <v>0.85176167498921518</v>
-      </c>
-      <c r="H3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I3" t="s">
-        <v>92</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" t="s">
-        <v>67</v>
-      </c>
-      <c r="L3" t="s">
-        <v>93</v>
+      <c r="J3">
+        <v>1.0188</v>
+      </c>
+      <c r="K3">
+        <v>1.88</v>
+      </c>
+      <c r="L3">
+        <v>0.869684112228528</v>
       </c>
       <c r="M3">
-        <v>2.4</v>
+        <v>0.18</v>
       </c>
       <c r="N3">
-        <v>5.8</v>
+        <v>3.58</v>
       </c>
     </row>
   </sheetData>
@@ -2267,19 +2350,19 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:N4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>63</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>77</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>78</v>
@@ -2315,136 +2398,136 @@
         <v>88</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2">
         <v>2024</v>
       </c>
-      <c r="B2">
+      <c r="C2">
         <v>2025</v>
       </c>
-      <c r="C2">
-        <v>4</v>
-      </c>
-      <c r="D2">
-        <v>0.9</v>
+      <c r="D2" t="s">
+        <v>89</v>
       </c>
       <c r="E2">
-        <v>1.0088999999999999</v>
-      </c>
-      <c r="F2">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I2">
         <v>11</v>
       </c>
-      <c r="G2">
-        <v>1.0078197863384679</v>
-      </c>
-      <c r="H2" t="s">
-        <v>89</v>
-      </c>
-      <c r="I2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J2" t="s">
+      <c r="J2">
+        <v>1.0149</v>
+      </c>
+      <c r="K2">
+        <v>1.49</v>
+      </c>
+      <c r="L2">
+        <v>1.323998280676608</v>
+      </c>
+      <c r="M2">
+        <v>-1.11</v>
+      </c>
+      <c r="N2">
+        <v>4.09</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
         <v>20</v>
       </c>
-      <c r="K2" t="s">
-        <v>67</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="B3">
+        <v>2025</v>
+      </c>
+      <c r="C3">
+        <v>2026</v>
+      </c>
+      <c r="D3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E3">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G3" t="s">
         <v>93</v>
       </c>
-      <c r="M2">
-        <v>-1.1000000000000001</v>
-      </c>
-      <c r="N2">
-        <v>2.9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>2025</v>
-      </c>
-      <c r="B3">
+      <c r="H3" t="s">
+        <v>91</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3">
+        <v>1.0188</v>
+      </c>
+      <c r="K3">
+        <v>1.88</v>
+      </c>
+      <c r="L3">
+        <v>0.869684112228528</v>
+      </c>
+      <c r="M3">
+        <v>0.18</v>
+      </c>
+      <c r="N3">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>2024</v>
+      </c>
+      <c r="C4">
         <v>2026</v>
       </c>
-      <c r="C3">
-        <v>4</v>
-      </c>
-      <c r="D3">
-        <v>4.0999999999999996</v>
-      </c>
-      <c r="E3">
-        <v>1.0407999999999999</v>
-      </c>
-      <c r="F3">
-        <v>10</v>
-      </c>
-      <c r="G3">
-        <v>0.85176167498921518</v>
-      </c>
-      <c r="H3" t="s">
-        <v>89</v>
-      </c>
-      <c r="I3" t="s">
-        <v>92</v>
-      </c>
-      <c r="J3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" t="s">
-        <v>67</v>
-      </c>
-      <c r="L3" t="s">
+      <c r="D4" t="s">
+        <v>94</v>
+      </c>
+      <c r="E4">
+        <v>7</v>
+      </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
+      <c r="G4" t="s">
         <v>93</v>
       </c>
-      <c r="M3">
-        <v>2.4</v>
-      </c>
-      <c r="N3">
-        <v>5.8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2024</v>
-      </c>
-      <c r="B4">
-        <v>2026</v>
-      </c>
-      <c r="C4">
-        <v>4</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-      <c r="E4">
-        <v>1.0500631199999999</v>
-      </c>
-      <c r="F4">
+      <c r="H4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I4">
         <v>11</v>
       </c>
-      <c r="G4">
-        <v>1.356029367955639</v>
-      </c>
-      <c r="H4" t="s">
-        <v>94</v>
-      </c>
-      <c r="I4" t="s">
-        <v>95</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K4" t="s">
-        <v>67</v>
-      </c>
-      <c r="L4" t="s">
-        <v>93</v>
+      <c r="J4">
+        <v>1.034</v>
+      </c>
+      <c r="K4">
+        <v>3.4</v>
+      </c>
+      <c r="L4">
+        <v>1.612046198451599</v>
       </c>
       <c r="M4">
-        <v>2.2999999999999998</v>
+        <v>0.24</v>
       </c>
       <c r="N4">
-        <v>7.7</v>
+        <v>6.56</v>
       </c>
     </row>
   </sheetData>
@@ -2453,257 +2536,380 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:M6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:M9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="10" max="10" width="20.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="J1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>63</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13">
       <c r="A2">
-        <v>1.0334894475519141</v>
+        <v>2025</v>
       </c>
       <c r="B2">
-        <v>3.3489447551913631</v>
-      </c>
-      <c r="C2">
+        <v>12</v>
+      </c>
+      <c r="C2" s="2">
+        <v>45992</v>
+      </c>
+      <c r="D2" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F2">
+        <v>1.0335</v>
+      </c>
+      <c r="G2">
+        <v>3.35</v>
+      </c>
+      <c r="H2">
+        <v>0.8</v>
+      </c>
+      <c r="I2">
+        <v>5.9</v>
+      </c>
+      <c r="J2">
         <v>8</v>
       </c>
-      <c r="D2">
-        <v>6.9615502771762756</v>
-      </c>
-      <c r="E2">
-        <v>2.804328922588307</v>
-      </c>
-      <c r="F2">
-        <v>1.062859770263745</v>
-      </c>
-      <c r="G2">
-        <v>0.8</v>
-      </c>
-      <c r="H2">
-        <v>5.9</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="K2">
+        <v>7</v>
+      </c>
+      <c r="L2">
+        <v>2.8</v>
+      </c>
+      <c r="M2">
+        <v>1.06</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3">
+        <v>2026</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46023</v>
+      </c>
+      <c r="D3" t="s">
         <v>103</v>
       </c>
-      <c r="J2" s="2">
-        <v>45992</v>
-      </c>
-      <c r="K2">
-        <v>12</v>
-      </c>
-      <c r="L2">
-        <v>2025</v>
-      </c>
-      <c r="M2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>1.0357387742376321</v>
-      </c>
-      <c r="B3">
-        <v>3.5738774237632498</v>
-      </c>
-      <c r="C3">
+      <c r="E3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3">
+        <v>1.0357</v>
+      </c>
+      <c r="G3">
+        <v>3.57</v>
+      </c>
+      <c r="H3">
+        <v>0.9</v>
+      </c>
+      <c r="I3">
+        <v>6.3</v>
+      </c>
+      <c r="J3">
         <v>8</v>
       </c>
-      <c r="D3">
-        <v>6.9615502771762756</v>
-      </c>
-      <c r="E3">
-        <v>3.0093285309362048</v>
-      </c>
-      <c r="F3">
-        <v>1.140556018688021</v>
-      </c>
-      <c r="G3">
-        <v>0.9</v>
-      </c>
-      <c r="H3">
-        <v>6.3</v>
-      </c>
-      <c r="I3" t="s">
-        <v>105</v>
-      </c>
-      <c r="J3" s="2">
-        <v>46023</v>
-      </c>
       <c r="K3">
+        <v>7</v>
+      </c>
+      <c r="L3">
+        <v>3.01</v>
+      </c>
+      <c r="M3">
+        <v>1.14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4">
+        <v>2026</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46054</v>
+      </c>
+      <c r="D4" t="s">
+        <v>103</v>
+      </c>
+      <c r="E4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F4">
+        <v>1.0388</v>
+      </c>
+      <c r="G4">
+        <v>3.88</v>
+      </c>
+      <c r="H4">
         <v>1</v>
       </c>
-      <c r="L3">
+      <c r="I4">
+        <v>6.7</v>
+      </c>
+      <c r="J4">
+        <v>8</v>
+      </c>
+      <c r="K4">
+        <v>7</v>
+      </c>
+      <c r="L4">
+        <v>3.2</v>
+      </c>
+      <c r="M4">
+        <v>1.21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5">
         <v>2026</v>
       </c>
-      <c r="M3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1.038780409927424</v>
-      </c>
-      <c r="B4">
-        <v>3.878040992742426</v>
-      </c>
-      <c r="C4">
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46082</v>
+      </c>
+      <c r="D5" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5">
+        <v>1.0426</v>
+      </c>
+      <c r="G5">
+        <v>4.26</v>
+      </c>
+      <c r="H5">
+        <v>1.2</v>
+      </c>
+      <c r="I5">
+        <v>7.4</v>
+      </c>
+      <c r="J5">
         <v>8</v>
       </c>
-      <c r="D4">
-        <v>6.9615502771762756</v>
-      </c>
-      <c r="E4">
-        <v>3.2044419398502568</v>
-      </c>
-      <c r="F4">
-        <v>1.2145053301626401</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-      <c r="H4">
-        <v>6.7</v>
-      </c>
-      <c r="I4" t="s">
-        <v>106</v>
-      </c>
-      <c r="J4" s="2">
-        <v>46054</v>
-      </c>
-      <c r="K4">
-        <v>2</v>
-      </c>
-      <c r="L4">
+      <c r="K5">
+        <v>7</v>
+      </c>
+      <c r="L5">
+        <v>3.45</v>
+      </c>
+      <c r="M5">
+        <v>1.31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13">
+      <c r="A6">
         <v>2026</v>
       </c>
-      <c r="M4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>1.0426430399660049</v>
-      </c>
-      <c r="B5">
-        <v>4.2643039966004936</v>
-      </c>
-      <c r="C5">
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46113</v>
+      </c>
+      <c r="D6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E6" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6">
+        <v>1.0481</v>
+      </c>
+      <c r="G6">
+        <v>4.81</v>
+      </c>
+      <c r="H6">
+        <v>1.6</v>
+      </c>
+      <c r="I6">
         <v>8</v>
       </c>
-      <c r="D5">
-        <v>6.9615502771762756</v>
-      </c>
-      <c r="E5">
-        <v>3.453201038408007</v>
-      </c>
-      <c r="F5">
-        <v>1.308786723552142</v>
-      </c>
-      <c r="G5">
-        <v>1.2</v>
-      </c>
-      <c r="H5">
-        <v>7.4</v>
-      </c>
-      <c r="I5" t="s">
-        <v>107</v>
-      </c>
-      <c r="J5" s="2">
-        <v>46082</v>
-      </c>
-      <c r="K5">
-        <v>3</v>
-      </c>
-      <c r="L5">
+      <c r="J6">
+        <v>8</v>
+      </c>
+      <c r="K6">
+        <v>7</v>
+      </c>
+      <c r="L6">
+        <v>3.57</v>
+      </c>
+      <c r="M6">
+        <v>1.35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13">
+      <c r="A7">
         <v>2026</v>
       </c>
-      <c r="M5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>1.048118973357447</v>
-      </c>
-      <c r="B6">
-        <v>4.8118973357447414</v>
-      </c>
-      <c r="C6">
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46143</v>
+      </c>
+      <c r="D7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E7" t="s">
+        <v>109</v>
+      </c>
+      <c r="F7">
+        <v>1.0482</v>
+      </c>
+      <c r="G7">
+        <v>4.82</v>
+      </c>
+      <c r="H7">
+        <v>1.5</v>
+      </c>
+      <c r="I7">
+        <v>8.1</v>
+      </c>
+      <c r="J7">
         <v>8</v>
       </c>
-      <c r="D6">
-        <v>6.9615502771762756</v>
-      </c>
-      <c r="E6">
-        <v>3.5678607777489888</v>
-      </c>
-      <c r="F6">
-        <v>1.352243546049974</v>
-      </c>
-      <c r="G6">
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>3.72</v>
+      </c>
+      <c r="M7">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13">
+      <c r="A8">
+        <v>2026</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" s="2">
+        <v>46174</v>
+      </c>
+      <c r="D8" t="s">
+        <v>103</v>
+      </c>
+      <c r="E8" t="s">
+        <v>110</v>
+      </c>
+      <c r="F8">
+        <v>1.0505</v>
+      </c>
+      <c r="G8">
+        <v>5.05</v>
+      </c>
+      <c r="H8">
         <v>1.6</v>
       </c>
-      <c r="H6">
+      <c r="I8">
+        <v>8.5</v>
+      </c>
+      <c r="J8">
         <v>8</v>
       </c>
-      <c r="I6" t="s">
-        <v>108</v>
-      </c>
-      <c r="J6" s="2">
-        <v>46113</v>
-      </c>
-      <c r="K6">
-        <v>4</v>
-      </c>
-      <c r="L6">
+      <c r="K8">
+        <v>7</v>
+      </c>
+      <c r="L8">
+        <v>3.81</v>
+      </c>
+      <c r="M8">
+        <v>1.45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13">
+      <c r="A9">
         <v>2026</v>
       </c>
-      <c r="M6" t="s">
-        <v>104</v>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46204</v>
+      </c>
+      <c r="D9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E9" t="s">
+        <v>111</v>
+      </c>
+      <c r="F9">
+        <v>1.0484</v>
+      </c>
+      <c r="G9">
+        <v>4.84</v>
+      </c>
+      <c r="H9">
+        <v>1.4</v>
+      </c>
+      <c r="I9">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="J9">
+        <v>8</v>
+      </c>
+      <c r="K9">
+        <v>7</v>
+      </c>
+      <c r="L9">
+        <v>3.82</v>
+      </c>
+      <c r="M9">
+        <v>1.45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>